<commit_message>
Add executive synthesis (SCR + MoM inflection mapping) and visual-proof placeholder slide
Adds an Executive_Synthesis sheet (SCR framework, MoM inflection mapping
across zones from validated series, and an explicit list of source data
needed for the velocity/distribution quadrant, opportunity-gap valuation,
and stock-productivity asks that current NSV-only sources can't support)
plus a placeholder Visual Proof slide (State + Chain banner boxes) since
no image source was available to pull execution photos automatically.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018SEDFnDPfSpnh1TqXh82kk
</commit_message>
<xml_diff>
--- a/MT_Offtake_Primary_Jun26_Working_CORRECTED.xlsx
+++ b/MT_Offtake_Primary_Jun26_Working_CORRECTED.xlsx
@@ -4,24 +4,25 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="READ_ME" sheetId="1" r:id="rId1"/>
-    <sheet name="Corrections_Impact" sheetId="2" r:id="rId2"/>
-    <sheet name="KPI_Dashboard" sheetId="3" r:id="rId3"/>
-    <sheet name="Q1_FY27_Scorecard" sheetId="4" r:id="rId4"/>
-    <sheet name="Zone_Summary" sheetId="5" r:id="rId5"/>
-    <sheet name="Chain_Summary" sheetId="6" r:id="rId6"/>
-    <sheet name="Brand_SubCat_Summary" sheetId="7" r:id="rId7"/>
-    <sheet name="Pack_Hero" sheetId="8" r:id="rId8"/>
-    <sheet name="Primary_Summary" sheetId="9" r:id="rId9"/>
-    <sheet name="May26_External_Workings" sheetId="10" r:id="rId10"/>
-    <sheet name="Slide_Map" sheetId="11" r:id="rId11"/>
-    <sheet name="Offtake_Chain_Zone" sheetId="12" r:id="rId12"/>
-    <sheet name="Offtake_Brand_SubCat_Zone" sheetId="13" r:id="rId13"/>
-    <sheet name="Offtake_Qtr_Chain_Zone" sheetId="14" r:id="rId14"/>
-    <sheet name="Zone_Brand_Qtr" sheetId="15" r:id="rId15"/>
-    <sheet name="Primary_Zone_Chain" sheetId="16" r:id="rId16"/>
-    <sheet name="Primary_Brand_Monthly" sheetId="17" r:id="rId17"/>
+    <sheet name="Executive_Synthesis" sheetId="2" r:id="rId2"/>
+    <sheet name="Corrections_Impact" sheetId="3" r:id="rId3"/>
+    <sheet name="KPI_Dashboard" sheetId="4" r:id="rId4"/>
+    <sheet name="Q1_FY27_Scorecard" sheetId="5" r:id="rId5"/>
+    <sheet name="Zone_Summary" sheetId="6" r:id="rId6"/>
+    <sheet name="Chain_Summary" sheetId="7" r:id="rId7"/>
+    <sheet name="Brand_SubCat_Summary" sheetId="8" r:id="rId8"/>
+    <sheet name="Pack_Hero" sheetId="9" r:id="rId9"/>
+    <sheet name="Primary_Summary" sheetId="10" r:id="rId10"/>
+    <sheet name="May26_External_Workings" sheetId="11" r:id="rId11"/>
+    <sheet name="Slide_Map" sheetId="12" r:id="rId12"/>
+    <sheet name="Offtake_Chain_Zone" sheetId="13" r:id="rId13"/>
+    <sheet name="Offtake_Brand_SubCat_Zone" sheetId="14" r:id="rId14"/>
+    <sheet name="Offtake_Qtr_Chain_Zone" sheetId="15" r:id="rId15"/>
+    <sheet name="Zone_Brand_Qtr" sheetId="16" r:id="rId16"/>
+    <sheet name="Primary_Zone_Chain" sheetId="17" r:id="rId17"/>
+    <sheet name="Primary_Brand_Monthly" sheetId="18" r:id="rId18"/>
   </sheets>
-  <calcPr calcId="199999" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -551,6 +552,974 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:R44"/>
+  <cols>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" customWidth="1"/>
+    <col min="7" max="7" width="10.83203125" customWidth="1"/>
+    <col min="8" max="8" width="10.83203125" customWidth="1"/>
+    <col min="9" max="9" width="10.83203125" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="10.83203125" customWidth="1"/>
+    <col min="13" max="13" width="10.83203125" customWidth="1"/>
+    <col min="14" max="14" width="10.83203125" customWidth="1"/>
+    <col min="15" max="15" width="10.83203125" customWidth="1"/>
+    <col min="16" max="16" width="10.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>PRIMARY (SELL-IN) SUMMARY — Jun'26 &amp; Q1 FY27 — ₹ Lacs</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Source: Primary_Zone_Chain (chain-level, ₹ Lacs) &amp; Primary_Brand_Monthly (brand-level, ₹). Live formulas.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Month</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Apr-25</v>
+      </c>
+      <c r="C4" t="str">
+        <v>May-25</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Jun-25</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Jul-25</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Aug-25</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Sep-25</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Oct-25</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Nov-25</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Dec-25</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Jan-26</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Feb-26</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Mar-26</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Apr-26</v>
+      </c>
+      <c r="O4" t="str">
+        <v>May-26</v>
+      </c>
+      <c r="P4" t="str">
+        <v>Jun-26</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Primary NSV total</v>
+      </c>
+      <c r="B5" s="1">
+        <f>SUM(Primary_Zone_Chain!D2:D200)</f>
+      </c>
+      <c r="C5" s="1">
+        <f>SUM(Primary_Zone_Chain!E2:E200)</f>
+      </c>
+      <c r="D5" s="1">
+        <f>SUM(Primary_Zone_Chain!F2:F200)</f>
+      </c>
+      <c r="E5" s="1">
+        <f>SUM(Primary_Zone_Chain!G2:G200)</f>
+      </c>
+      <c r="F5" s="1">
+        <f>SUM(Primary_Zone_Chain!H2:H200)</f>
+      </c>
+      <c r="G5" s="1">
+        <f>SUM(Primary_Zone_Chain!I2:I200)</f>
+      </c>
+      <c r="H5" s="1">
+        <f>SUM(Primary_Zone_Chain!J2:J200)</f>
+      </c>
+      <c r="I5" s="1">
+        <f>SUM(Primary_Zone_Chain!K2:K200)</f>
+      </c>
+      <c r="J5" s="1">
+        <f>SUM(Primary_Zone_Chain!L2:L200)</f>
+      </c>
+      <c r="K5" s="1">
+        <f>SUM(Primary_Zone_Chain!M2:M200)</f>
+      </c>
+      <c r="L5" s="1">
+        <f>SUM(Primary_Zone_Chain!N2:N200)</f>
+      </c>
+      <c r="M5" s="1">
+        <f>SUM(Primary_Zone_Chain!O2:O200)</f>
+      </c>
+      <c r="N5" s="1">
+        <f>SUM(Primary_Zone_Chain!P2:P200)</f>
+      </c>
+      <c r="O5" s="1">
+        <f>SUM(Primary_Zone_Chain!Q2:Q200)</f>
+      </c>
+      <c r="P5" s="1">
+        <f>SUM(Primary_Zone_Chain!R2:R200)</f>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>MoM %</v>
+      </c>
+      <c r="C6" s="4">
+        <f>C5/B5-1</f>
+      </c>
+      <c r="D6" s="4">
+        <f>D5/C5-1</f>
+      </c>
+      <c r="E6" s="4">
+        <f>E5/D5-1</f>
+      </c>
+      <c r="F6" s="4">
+        <f>F5/E5-1</f>
+      </c>
+      <c r="G6" s="4">
+        <f>G5/F5-1</f>
+      </c>
+      <c r="H6" s="4">
+        <f>H5/G5-1</f>
+      </c>
+      <c r="I6" s="4">
+        <f>I5/H5-1</f>
+      </c>
+      <c r="J6" s="4">
+        <f>J5/I5-1</f>
+      </c>
+      <c r="K6" s="4">
+        <f>K5/J5-1</f>
+      </c>
+      <c r="L6" s="4">
+        <f>L5/K5-1</f>
+      </c>
+      <c r="M6" s="4">
+        <f>M5/L5-1</f>
+      </c>
+      <c r="N6" s="4">
+        <f>N5/M5-1</f>
+      </c>
+      <c r="O6" s="4">
+        <f>O5/N5-1</f>
+      </c>
+      <c r="P6" s="4">
+        <f>P5/O5-1</f>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>YoY %</v>
+      </c>
+      <c r="N7" s="4">
+        <f>N5/B5-1</f>
+      </c>
+      <c r="O7" s="4">
+        <f>O5/C5-1</f>
+      </c>
+      <c r="P7" s="4">
+        <f>P5/D5-1</f>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>HEADLINES</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Jun'26 Primary (₹ Cr)</v>
+      </c>
+      <c r="C10" s="5">
+        <f>P5/100</f>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>MoM %</v>
+      </c>
+      <c r="C11" s="4">
+        <f>P5/O5-1</f>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>GOLY % (vs Jun'25)</v>
+      </c>
+      <c r="C12" s="4">
+        <f>P5/D5-1</f>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Q1 FY27 (₹ Cr)</v>
+      </c>
+      <c r="C13" s="5">
+        <f>SUM(N5:P5)/100</f>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Q1 FY26 (₹ Cr)</v>
+      </c>
+      <c r="C14" s="5">
+        <f>SUM(B5:D5)/100</f>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Q1 growth %</v>
+      </c>
+      <c r="C15" s="4">
+        <f>SUM(N5:P5)/SUM(B5:D5)-1</f>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>BY CHAIN (top primary billings)</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v/>
+      </c>
+      <c r="B18" t="str">
+        <v>Jun-25</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Apr-26</v>
+      </c>
+      <c r="D18" t="str">
+        <v>May-26</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Jun-26</v>
+      </c>
+      <c r="F18" t="str">
+        <v>MoM %</v>
+      </c>
+      <c r="G18" t="str">
+        <v>GOLY %</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Q1 FY26</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Q1 FY27</v>
+      </c>
+      <c r="J18" t="str">
+        <v>Q1 Gr %</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>D-Mart</v>
+      </c>
+      <c r="B19" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="C19" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!P:P)</f>
+      </c>
+      <c r="D19" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!Q:Q)</f>
+      </c>
+      <c r="E19" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="F19" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!Q:Q)-1</f>
+      </c>
+      <c r="G19" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!F:F)-1</f>
+      </c>
+      <c r="H19" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="I19" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="J19" s="4">
+        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!F:F))-1</f>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Reliance Retail</v>
+      </c>
+      <c r="B20" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="C20" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!P:P)</f>
+      </c>
+      <c r="D20" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!Q:Q)</f>
+      </c>
+      <c r="E20" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="F20" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!Q:Q)-1</f>
+      </c>
+      <c r="G20" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!F:F)-1</f>
+      </c>
+      <c r="H20" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="I20" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="J20" s="4">
+        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!F:F))-1</f>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Apollo Healthco</v>
+      </c>
+      <c r="B21" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="C21" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!P:P)</f>
+      </c>
+      <c r="D21" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!Q:Q)</f>
+      </c>
+      <c r="E21" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="F21" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!Q:Q)-1</f>
+      </c>
+      <c r="G21" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!F:F)-1</f>
+      </c>
+      <c r="H21" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="I21" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="J21" s="4">
+        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!F:F))-1</f>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Lulu</v>
+      </c>
+      <c r="B22" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="C22" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!P:P)</f>
+      </c>
+      <c r="D22" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!Q:Q)</f>
+      </c>
+      <c r="E22" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="F22" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!Q:Q)-1</f>
+      </c>
+      <c r="G22" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!F:F)-1</f>
+      </c>
+      <c r="H22" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="I22" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="J22" s="4">
+        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!F:F))-1</f>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Wellness Forever</v>
+      </c>
+      <c r="B23" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="C23" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!P:P)</f>
+      </c>
+      <c r="D23" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!Q:Q)</f>
+      </c>
+      <c r="E23" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="F23" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!Q:Q)-1</f>
+      </c>
+      <c r="G23" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!F:F)-1</f>
+      </c>
+      <c r="H23" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="I23" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="J23" s="4">
+        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!F:F))-1</f>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>H&amp;G</v>
+      </c>
+      <c r="B24" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="C24" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!P:P)</f>
+      </c>
+      <c r="D24" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!Q:Q)</f>
+      </c>
+      <c r="E24" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="F24" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!Q:Q)-1</f>
+      </c>
+      <c r="G24" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!F:F)-1</f>
+      </c>
+      <c r="H24" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="I24" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="J24" s="4">
+        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!F:F))-1</f>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>RMT-Sancus</v>
+      </c>
+      <c r="B25" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="C25" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!P:P)</f>
+      </c>
+      <c r="D25" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!Q:Q)</f>
+      </c>
+      <c r="E25" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="F25" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!Q:Q)-1</f>
+      </c>
+      <c r="G25" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!F:F)-1</f>
+      </c>
+      <c r="H25" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="I25" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="J25" s="4">
+        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!F:F))-1</f>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>VMM</v>
+      </c>
+      <c r="B26" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="C26" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!P:P)</f>
+      </c>
+      <c r="D26" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!Q:Q)</f>
+      </c>
+      <c r="E26" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="F26" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!Q:Q)-1</f>
+      </c>
+      <c r="G26" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!F:F)-1</f>
+      </c>
+      <c r="H26" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="I26" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="J26" s="4">
+        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!F:F))-1</f>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>More Retail</v>
+      </c>
+      <c r="B27" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="C27" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!P:P)</f>
+      </c>
+      <c r="D27" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!Q:Q)</f>
+      </c>
+      <c r="E27" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="F27" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!Q:Q)-1</f>
+      </c>
+      <c r="G27" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!F:F)-1</f>
+      </c>
+      <c r="H27" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="I27" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="J27" s="4">
+        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!F:F))-1</f>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Nykaa SS(fsn)</v>
+      </c>
+      <c r="B28" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="C28" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!P:P)</f>
+      </c>
+      <c r="D28" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!Q:Q)</f>
+      </c>
+      <c r="E28" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="F28" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!Q:Q)-1</f>
+      </c>
+      <c r="G28" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!F:F)-1</f>
+      </c>
+      <c r="H28" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="I28" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="J28" s="4">
+        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!F:F))-1</f>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Metro-CNC-RRL</v>
+      </c>
+      <c r="B29" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="C29" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!P:P)</f>
+      </c>
+      <c r="D29" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!Q:Q)</f>
+      </c>
+      <c r="E29" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="F29" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!Q:Q)-1</f>
+      </c>
+      <c r="G29" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!F:F)-1</f>
+      </c>
+      <c r="H29" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="I29" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="J29" s="4">
+        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!F:F))-1</f>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Frankross</v>
+      </c>
+      <c r="B30" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="C30" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!P:P)</f>
+      </c>
+      <c r="D30" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!Q:Q)</f>
+      </c>
+      <c r="E30" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="F30" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!Q:Q)-1</f>
+      </c>
+      <c r="G30" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!F:F)-1</f>
+      </c>
+      <c r="H30" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="I30" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="J30" s="4">
+        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!F:F))-1</f>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Spencer</v>
+      </c>
+      <c r="B31" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="C31" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!P:P)</f>
+      </c>
+      <c r="D31" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!Q:Q)</f>
+      </c>
+      <c r="E31" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="F31" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!Q:Q)-1</f>
+      </c>
+      <c r="G31" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!F:F)-1</f>
+      </c>
+      <c r="H31" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="I31" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="J31" s="4">
+        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!F:F))-1</f>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Walmart CNC</v>
+      </c>
+      <c r="B32" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="C32" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!P:P)</f>
+      </c>
+      <c r="D32" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!Q:Q)</f>
+      </c>
+      <c r="E32" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="F32" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!Q:Q)-1</f>
+      </c>
+      <c r="G32" s="4">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!F:F)-1</f>
+      </c>
+      <c r="H32" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!F:F)</f>
+      </c>
+      <c r="I32" s="1">
+        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!R:R)</f>
+      </c>
+      <c r="J32" s="4">
+        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!F:F))-1</f>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>BY BRAND (₹ Lacs, from Primary_Brand_Monthly ₹)</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v/>
+      </c>
+      <c r="B35" t="str">
+        <v>Jun-25</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Apr-26</v>
+      </c>
+      <c r="D35" t="str">
+        <v>May-26</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Jun-26</v>
+      </c>
+      <c r="F35" t="str">
+        <v>MoM %</v>
+      </c>
+      <c r="G35" t="str">
+        <v>GOLY %</v>
+      </c>
+      <c r="H35" t="str">
+        <v>Q1 FY26</v>
+      </c>
+      <c r="I35" t="str">
+        <v>Q1 FY27</v>
+      </c>
+      <c r="J35" t="str">
+        <v>Q1 Gr %</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Mamaearth (MT)</v>
+      </c>
+      <c r="B36" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="C36" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="D36" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="E36" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="F36" s="4">
+        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
+      </c>
+      <c r="G36" s="4">
+        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
+      </c>
+      <c r="H36" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="I36" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="J36" s="4">
+        <f>(SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000)/(SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000)-1</f>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>The Derma Co. (MT)</v>
+      </c>
+      <c r="B37" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="C37" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="D37" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="E37" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="F37" s="4">
+        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
+      </c>
+      <c r="G37" s="4">
+        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
+      </c>
+      <c r="H37" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="I37" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="J37" s="4">
+        <f>(SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000)/(SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000)-1</f>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Aqualogica (MT)</v>
+      </c>
+      <c r="B38" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="C38" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="D38" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="E38" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="F38" s="4">
+        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
+      </c>
+      <c r="G38" s="4">
+        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
+      </c>
+      <c r="H38" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="I38" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="J38" s="4">
+        <f>(SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000)/(SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000)-1</f>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Mamaearth (EB2B)</v>
+      </c>
+      <c r="B39" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="C39" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="D39" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="E39" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="F39" s="4">
+        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
+      </c>
+      <c r="G39" s="4">
+        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
+      </c>
+      <c r="H39" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="I39" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="J39" s="4">
+        <f>(SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000)/(SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000)-1</f>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>The Derma Co. (EB2B)</v>
+      </c>
+      <c r="B40" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="C40" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="D40" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="E40" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="F40" s="4">
+        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
+      </c>
+      <c r="G40" s="4">
+        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
+      </c>
+      <c r="H40" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="I40" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="J40" s="4">
+        <f>(SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000)/(SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000)-1</f>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>ALL-IN GRAND TOTAL</v>
+      </c>
+      <c r="B41" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="C41" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="D41" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="E41" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="F41" s="4">
+        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
+      </c>
+      <c r="G41" s="4">
+        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
+      </c>
+      <c r="H41" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="I41" s="1">
+        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
+      </c>
+      <c r="J41" s="4">
+        <f>(SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000)/(SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000)-1</f>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:R44"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J20"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
@@ -785,7 +1754,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D18"/>
   <cols>
@@ -1054,7 +2023,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:T83"/>
   <cols>
@@ -5678,7 +6647,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:U229"/>
   <cols>
@@ -20318,7 +21287,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P93"/>
   <cols>
@@ -24214,7 +25183,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Q36"/>
   <cols>
@@ -25900,7 +26869,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:T109"/>
   <cols>
@@ -30885,7 +31854,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:W31"/>
   <cols>
@@ -32827,6 +33796,219 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D26"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="60.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>EXECUTIVE SYNTHESIS — Q1 FY26-27 (Apr-Jun'26) — SCR FRAMEWORK</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Brand | Category | SKU anchor: Mamaearth + The Derma Co. | Face Care / Hair Care / Sun Care | Portfolio-wide</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>SITUATION</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Q1 FY27 NSV hit ₹11,438.7L vs ₹6,986.0L in Q1 FY26 — up 63.7% YoY, led by West and Derma Co.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>COMPLICATION</v>
+      </c>
+      <c r="B5" t="str">
+        <v>June momentum cooled everywhere at once — every zone decelerated MoM after a May peak (-5.0% co. wide).</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>RESOLUTION</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Protect May's pipeline-fill gains by shifting focus to June sell-through; re-forecast July off L3M avg (₹3,615L), not May peak.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>MoM INFLECTION MAPPING (real, from 15-month series — no fabricated inputs)</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Every one of the 6 zones shows the identical inflection shape: acceleration into May-26 (peak MoM), then sharp deceleration in June-26.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>This is a company-wide pattern, most consistent with a May primary pipeline-fill/stockist-loading effect rather than a genuine June demand drop.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Zone</v>
+      </c>
+      <c r="B12" t="str">
+        <v>May MoM %</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Jun MoM %</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Read</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>EAST</v>
+      </c>
+      <c r="B13">
+        <v>11.4</v>
+      </c>
+      <c r="C13">
+        <v>-6.7</v>
+      </c>
+      <c r="D13" t="str">
+        <v>May peak -&gt; Jun correction</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>NORTH</v>
+      </c>
+      <c r="B14">
+        <v>3.7</v>
+      </c>
+      <c r="C14">
+        <v>-8.2</v>
+      </c>
+      <c r="D14" t="str">
+        <v>May peak -&gt; Jun correction</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>SOUTH-1</v>
+      </c>
+      <c r="B15">
+        <v>15.1</v>
+      </c>
+      <c r="C15">
+        <v>-4.6</v>
+      </c>
+      <c r="D15" t="str">
+        <v>May peak -&gt; Jun correction</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>SOUTH-2</v>
+      </c>
+      <c r="B16">
+        <v>10.1</v>
+      </c>
+      <c r="C16">
+        <v>-3.1</v>
+      </c>
+      <c r="D16" t="str">
+        <v>May peak -&gt; Jun correction</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>WEST</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17">
+        <v>-0.7</v>
+      </c>
+      <c r="D17" t="str">
+        <v>May peak -&gt; Jun correction (mildest)</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>PAN INDIA</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Smallest zone, more volatile</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>DATA REQUIRED TO COMPLETE REMAINING ASKS (flagged, not fabricated — per no-dummy-data rule)</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Velocity-vs-Distribution Quadrant, Opportunity Gap Valuation, and Stock Productivity/Capital Efficiency need inputs our</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>source tables do not contain (sales NSV/volume only). To build these for real, please share:</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>1. Store count / active distribution points per chain per zone per month (Peak Throughput per store, Active Distribution Grid, Quadrant classification).</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>2. Monthly sales target/budget per zone or brand (Opportunity Gap Valuation = Target - Carrying Variance x Peak Throughput Velocity).</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>3. Inventory/stock-in-trade and shelf-space (bay/facing) allocation per chain (Stock Productivity &amp; Capital Efficiency).</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Once shared, these will be validated and added as formula-linked sheets/slides using the same process as the NSV corrections.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D26"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J30"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
@@ -33412,7 +34594,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Q30"/>
   <cols>
@@ -33827,7 +35009,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H33"/>
   <cols>
@@ -34271,7 +35453,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O21"/>
   <cols>
@@ -34635,7 +35817,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O41"/>
   <cols>
@@ -35819,7 +37001,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O19"/>
   <cols>
@@ -36393,7 +37575,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:N93"/>
   <cols>
@@ -40459,972 +41641,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:N93"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R44"/>
-  <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" customWidth="1"/>
-    <col min="9" max="9" width="10.83203125" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="10.83203125" customWidth="1"/>
-    <col min="13" max="13" width="10.83203125" customWidth="1"/>
-    <col min="14" max="14" width="10.83203125" customWidth="1"/>
-    <col min="15" max="15" width="10.83203125" customWidth="1"/>
-    <col min="16" max="16" width="10.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>PRIMARY (SELL-IN) SUMMARY — Jun'26 &amp; Q1 FY27 — ₹ Lacs</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Source: Primary_Zone_Chain (chain-level, ₹ Lacs) &amp; Primary_Brand_Monthly (brand-level, ₹). Live formulas.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Month</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Apr-25</v>
-      </c>
-      <c r="C4" t="str">
-        <v>May-25</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Jun-25</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Jul-25</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Aug-25</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Sep-25</v>
-      </c>
-      <c r="H4" t="str">
-        <v>Oct-25</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Nov-25</v>
-      </c>
-      <c r="J4" t="str">
-        <v>Dec-25</v>
-      </c>
-      <c r="K4" t="str">
-        <v>Jan-26</v>
-      </c>
-      <c r="L4" t="str">
-        <v>Feb-26</v>
-      </c>
-      <c r="M4" t="str">
-        <v>Mar-26</v>
-      </c>
-      <c r="N4" t="str">
-        <v>Apr-26</v>
-      </c>
-      <c r="O4" t="str">
-        <v>May-26</v>
-      </c>
-      <c r="P4" t="str">
-        <v>Jun-26</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Primary NSV total</v>
-      </c>
-      <c r="B5" s="1">
-        <f>SUM(Primary_Zone_Chain!D2:D200)</f>
-      </c>
-      <c r="C5" s="1">
-        <f>SUM(Primary_Zone_Chain!E2:E200)</f>
-      </c>
-      <c r="D5" s="1">
-        <f>SUM(Primary_Zone_Chain!F2:F200)</f>
-      </c>
-      <c r="E5" s="1">
-        <f>SUM(Primary_Zone_Chain!G2:G200)</f>
-      </c>
-      <c r="F5" s="1">
-        <f>SUM(Primary_Zone_Chain!H2:H200)</f>
-      </c>
-      <c r="G5" s="1">
-        <f>SUM(Primary_Zone_Chain!I2:I200)</f>
-      </c>
-      <c r="H5" s="1">
-        <f>SUM(Primary_Zone_Chain!J2:J200)</f>
-      </c>
-      <c r="I5" s="1">
-        <f>SUM(Primary_Zone_Chain!K2:K200)</f>
-      </c>
-      <c r="J5" s="1">
-        <f>SUM(Primary_Zone_Chain!L2:L200)</f>
-      </c>
-      <c r="K5" s="1">
-        <f>SUM(Primary_Zone_Chain!M2:M200)</f>
-      </c>
-      <c r="L5" s="1">
-        <f>SUM(Primary_Zone_Chain!N2:N200)</f>
-      </c>
-      <c r="M5" s="1">
-        <f>SUM(Primary_Zone_Chain!O2:O200)</f>
-      </c>
-      <c r="N5" s="1">
-        <f>SUM(Primary_Zone_Chain!P2:P200)</f>
-      </c>
-      <c r="O5" s="1">
-        <f>SUM(Primary_Zone_Chain!Q2:Q200)</f>
-      </c>
-      <c r="P5" s="1">
-        <f>SUM(Primary_Zone_Chain!R2:R200)</f>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>MoM %</v>
-      </c>
-      <c r="C6" s="4">
-        <f>C5/B5-1</f>
-      </c>
-      <c r="D6" s="4">
-        <f>D5/C5-1</f>
-      </c>
-      <c r="E6" s="4">
-        <f>E5/D5-1</f>
-      </c>
-      <c r="F6" s="4">
-        <f>F5/E5-1</f>
-      </c>
-      <c r="G6" s="4">
-        <f>G5/F5-1</f>
-      </c>
-      <c r="H6" s="4">
-        <f>H5/G5-1</f>
-      </c>
-      <c r="I6" s="4">
-        <f>I5/H5-1</f>
-      </c>
-      <c r="J6" s="4">
-        <f>J5/I5-1</f>
-      </c>
-      <c r="K6" s="4">
-        <f>K5/J5-1</f>
-      </c>
-      <c r="L6" s="4">
-        <f>L5/K5-1</f>
-      </c>
-      <c r="M6" s="4">
-        <f>M5/L5-1</f>
-      </c>
-      <c r="N6" s="4">
-        <f>N5/M5-1</f>
-      </c>
-      <c r="O6" s="4">
-        <f>O5/N5-1</f>
-      </c>
-      <c r="P6" s="4">
-        <f>P5/O5-1</f>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>YoY %</v>
-      </c>
-      <c r="N7" s="4">
-        <f>N5/B5-1</f>
-      </c>
-      <c r="O7" s="4">
-        <f>O5/C5-1</f>
-      </c>
-      <c r="P7" s="4">
-        <f>P5/D5-1</f>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>HEADLINES</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Jun'26 Primary (₹ Cr)</v>
-      </c>
-      <c r="C10" s="5">
-        <f>P5/100</f>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>MoM %</v>
-      </c>
-      <c r="C11" s="4">
-        <f>P5/O5-1</f>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>GOLY % (vs Jun'25)</v>
-      </c>
-      <c r="C12" s="4">
-        <f>P5/D5-1</f>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Q1 FY27 (₹ Cr)</v>
-      </c>
-      <c r="C13" s="5">
-        <f>SUM(N5:P5)/100</f>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Q1 FY26 (₹ Cr)</v>
-      </c>
-      <c r="C14" s="5">
-        <f>SUM(B5:D5)/100</f>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Q1 growth %</v>
-      </c>
-      <c r="C15" s="4">
-        <f>SUM(N5:P5)/SUM(B5:D5)-1</f>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>BY CHAIN (top primary billings)</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v/>
-      </c>
-      <c r="B18" t="str">
-        <v>Jun-25</v>
-      </c>
-      <c r="C18" t="str">
-        <v>Apr-26</v>
-      </c>
-      <c r="D18" t="str">
-        <v>May-26</v>
-      </c>
-      <c r="E18" t="str">
-        <v>Jun-26</v>
-      </c>
-      <c r="F18" t="str">
-        <v>MoM %</v>
-      </c>
-      <c r="G18" t="str">
-        <v>GOLY %</v>
-      </c>
-      <c r="H18" t="str">
-        <v>Q1 FY26</v>
-      </c>
-      <c r="I18" t="str">
-        <v>Q1 FY27</v>
-      </c>
-      <c r="J18" t="str">
-        <v>Q1 Gr %</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>D-Mart</v>
-      </c>
-      <c r="B19" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="C19" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!P:P)</f>
-      </c>
-      <c r="D19" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!Q:Q)</f>
-      </c>
-      <c r="E19" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="F19" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!Q:Q)-1</f>
-      </c>
-      <c r="G19" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!F:F)-1</f>
-      </c>
-      <c r="H19" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="I19" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="J19" s="4">
-        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"D-Mart",Primary_Zone_Chain!F:F))-1</f>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>Reliance Retail</v>
-      </c>
-      <c r="B20" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="C20" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!P:P)</f>
-      </c>
-      <c r="D20" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!Q:Q)</f>
-      </c>
-      <c r="E20" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="F20" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!Q:Q)-1</f>
-      </c>
-      <c r="G20" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!F:F)-1</f>
-      </c>
-      <c r="H20" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="I20" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="J20" s="4">
-        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Reliance Retail",Primary_Zone_Chain!F:F))-1</f>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>Apollo Healthco</v>
-      </c>
-      <c r="B21" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="C21" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!P:P)</f>
-      </c>
-      <c r="D21" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!Q:Q)</f>
-      </c>
-      <c r="E21" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="F21" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!Q:Q)-1</f>
-      </c>
-      <c r="G21" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!F:F)-1</f>
-      </c>
-      <c r="H21" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="I21" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="J21" s="4">
-        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Apollo Healthco",Primary_Zone_Chain!F:F))-1</f>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>Lulu</v>
-      </c>
-      <c r="B22" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="C22" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!P:P)</f>
-      </c>
-      <c r="D22" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!Q:Q)</f>
-      </c>
-      <c r="E22" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="F22" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!Q:Q)-1</f>
-      </c>
-      <c r="G22" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!F:F)-1</f>
-      </c>
-      <c r="H22" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="I22" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="J22" s="4">
-        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Lulu",Primary_Zone_Chain!F:F))-1</f>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>Wellness Forever</v>
-      </c>
-      <c r="B23" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="C23" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!P:P)</f>
-      </c>
-      <c r="D23" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!Q:Q)</f>
-      </c>
-      <c r="E23" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="F23" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!Q:Q)-1</f>
-      </c>
-      <c r="G23" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!F:F)-1</f>
-      </c>
-      <c r="H23" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="I23" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="J23" s="4">
-        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Wellness Forever",Primary_Zone_Chain!F:F))-1</f>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>H&amp;G</v>
-      </c>
-      <c r="B24" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="C24" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!P:P)</f>
-      </c>
-      <c r="D24" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!Q:Q)</f>
-      </c>
-      <c r="E24" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="F24" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!Q:Q)-1</f>
-      </c>
-      <c r="G24" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!F:F)-1</f>
-      </c>
-      <c r="H24" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="I24" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="J24" s="4">
-        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"H&amp;G",Primary_Zone_Chain!F:F))-1</f>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>RMT-Sancus</v>
-      </c>
-      <c r="B25" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="C25" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!P:P)</f>
-      </c>
-      <c r="D25" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!Q:Q)</f>
-      </c>
-      <c r="E25" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="F25" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!Q:Q)-1</f>
-      </c>
-      <c r="G25" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!F:F)-1</f>
-      </c>
-      <c r="H25" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="I25" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="J25" s="4">
-        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"RMT-Sancus",Primary_Zone_Chain!F:F))-1</f>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>VMM</v>
-      </c>
-      <c r="B26" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="C26" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!P:P)</f>
-      </c>
-      <c r="D26" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!Q:Q)</f>
-      </c>
-      <c r="E26" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="F26" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!Q:Q)-1</f>
-      </c>
-      <c r="G26" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!F:F)-1</f>
-      </c>
-      <c r="H26" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="I26" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="J26" s="4">
-        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"VMM",Primary_Zone_Chain!F:F))-1</f>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>More Retail</v>
-      </c>
-      <c r="B27" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="C27" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!P:P)</f>
-      </c>
-      <c r="D27" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!Q:Q)</f>
-      </c>
-      <c r="E27" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="F27" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!Q:Q)-1</f>
-      </c>
-      <c r="G27" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!F:F)-1</f>
-      </c>
-      <c r="H27" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="I27" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="J27" s="4">
-        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"More Retail",Primary_Zone_Chain!F:F))-1</f>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>Nykaa SS(fsn)</v>
-      </c>
-      <c r="B28" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="C28" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!P:P)</f>
-      </c>
-      <c r="D28" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!Q:Q)</f>
-      </c>
-      <c r="E28" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="F28" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!Q:Q)-1</f>
-      </c>
-      <c r="G28" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!F:F)-1</f>
-      </c>
-      <c r="H28" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="I28" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="J28" s="4">
-        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Nykaa SS(fsn)",Primary_Zone_Chain!F:F))-1</f>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>Metro-CNC-RRL</v>
-      </c>
-      <c r="B29" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="C29" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!P:P)</f>
-      </c>
-      <c r="D29" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!Q:Q)</f>
-      </c>
-      <c r="E29" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="F29" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!Q:Q)-1</f>
-      </c>
-      <c r="G29" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!F:F)-1</f>
-      </c>
-      <c r="H29" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="I29" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="J29" s="4">
-        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Metro-CNC-RRL",Primary_Zone_Chain!F:F))-1</f>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>Frankross</v>
-      </c>
-      <c r="B30" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="C30" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!P:P)</f>
-      </c>
-      <c r="D30" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!Q:Q)</f>
-      </c>
-      <c r="E30" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="F30" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!Q:Q)-1</f>
-      </c>
-      <c r="G30" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!F:F)-1</f>
-      </c>
-      <c r="H30" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="I30" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="J30" s="4">
-        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Frankross",Primary_Zone_Chain!F:F))-1</f>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>Spencer</v>
-      </c>
-      <c r="B31" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="C31" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!P:P)</f>
-      </c>
-      <c r="D31" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!Q:Q)</f>
-      </c>
-      <c r="E31" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="F31" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!Q:Q)-1</f>
-      </c>
-      <c r="G31" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!F:F)-1</f>
-      </c>
-      <c r="H31" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="I31" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="J31" s="4">
-        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Spencer",Primary_Zone_Chain!F:F))-1</f>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>Walmart CNC</v>
-      </c>
-      <c r="B32" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="C32" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!P:P)</f>
-      </c>
-      <c r="D32" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!Q:Q)</f>
-      </c>
-      <c r="E32" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="F32" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!Q:Q)-1</f>
-      </c>
-      <c r="G32" s="4">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!R:R)/SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!F:F)-1</f>
-      </c>
-      <c r="H32" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!F:F)</f>
-      </c>
-      <c r="I32" s="1">
-        <f>SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!R:R)</f>
-      </c>
-      <c r="J32" s="4">
-        <f>(SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!P:P)+SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!Q:Q)+SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!R:R))/(SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!D:D)+SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!E:E)+SUMIF(Primary_Zone_Chain!$C:$C,"Walmart CNC",Primary_Zone_Chain!F:F))-1</f>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>BY BRAND (₹ Lacs, from Primary_Brand_Monthly ₹)</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v/>
-      </c>
-      <c r="B35" t="str">
-        <v>Jun-25</v>
-      </c>
-      <c r="C35" t="str">
-        <v>Apr-26</v>
-      </c>
-      <c r="D35" t="str">
-        <v>May-26</v>
-      </c>
-      <c r="E35" t="str">
-        <v>Jun-26</v>
-      </c>
-      <c r="F35" t="str">
-        <v>MoM %</v>
-      </c>
-      <c r="G35" t="str">
-        <v>GOLY %</v>
-      </c>
-      <c r="H35" t="str">
-        <v>Q1 FY26</v>
-      </c>
-      <c r="I35" t="str">
-        <v>Q1 FY27</v>
-      </c>
-      <c r="J35" t="str">
-        <v>Q1 Gr %</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>Mamaearth (MT)</v>
-      </c>
-      <c r="B36" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="C36" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="D36" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="E36" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="F36" s="4">
-        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
-      </c>
-      <c r="G36" s="4">
-        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
-      </c>
-      <c r="H36" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="I36" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="J36" s="4">
-        <f>(SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000)/(SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000)-1</f>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>The Derma Co. (MT)</v>
-      </c>
-      <c r="B37" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="C37" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="D37" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="E37" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="F37" s="4">
-        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
-      </c>
-      <c r="G37" s="4">
-        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
-      </c>
-      <c r="H37" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="I37" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="J37" s="4">
-        <f>(SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000)/(SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000)-1</f>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="str">
-        <v>Aqualogica (MT)</v>
-      </c>
-      <c r="B38" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="C38" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="D38" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="E38" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="F38" s="4">
-        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
-      </c>
-      <c r="G38" s="4">
-        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
-      </c>
-      <c r="H38" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="I38" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="J38" s="4">
-        <f>(SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000)/(SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"MT",Primary_Brand_Monthly!$B:$B,"Aqualogica",Primary_Brand_Monthly!$C:$C,"ALL")/100000)-1</f>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="str">
-        <v>Mamaearth (EB2B)</v>
-      </c>
-      <c r="B39" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="C39" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="D39" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="E39" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="F39" s="4">
-        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
-      </c>
-      <c r="G39" s="4">
-        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
-      </c>
-      <c r="H39" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="I39" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="J39" s="4">
-        <f>(SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000)/(SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"Mamaearth",Primary_Brand_Monthly!$C:$C,"ALL")/100000)-1</f>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="str">
-        <v>The Derma Co. (EB2B)</v>
-      </c>
-      <c r="B40" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="C40" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="D40" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="E40" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="F40" s="4">
-        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
-      </c>
-      <c r="G40" s="4">
-        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
-      </c>
-      <c r="H40" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="I40" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="J40" s="4">
-        <f>(SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000)/(SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"Eb2b",Primary_Brand_Monthly!$B:$B,"The Derma Co.",Primary_Brand_Monthly!$C:$C,"ALL")/100000)-1</f>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="str">
-        <v>ALL-IN GRAND TOTAL</v>
-      </c>
-      <c r="B41" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="C41" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="D41" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="E41" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="F41" s="4">
-        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
-      </c>
-      <c r="G41" s="4">
-        <f>SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000/SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000-1</f>
-      </c>
-      <c r="H41" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="I41" s="1">
-        <f>SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000</f>
-      </c>
-      <c r="J41" s="4">
-        <f>(SUMIFS(Primary_Brand_Monthly!S:S,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!T:T,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!U:U,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000)/(SUMIFS(Primary_Brand_Monthly!G:G,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!H:H,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000+SUMIFS(Primary_Brand_Monthly!I:I,Primary_Brand_Monthly!$A:$A,"ALL",Primary_Brand_Monthly!$B:$B,"GRAND TOTAL",Primary_Brand_Monthly!$C:$C,"ALL")/100000)-1</f>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R44"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>